<commit_message>
Update menu data from menu novi 3.ods and regenerate PDF
</commit_message>
<xml_diff>
--- a/public/menu.xlsx
+++ b/public/menu.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E96"/>
+  <dimension ref="A1:E97"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1552,7 +1552,7 @@
         </is>
       </c>
       <c r="E45" t="n">
-        <v>350</v>
+        <v>400</v>
       </c>
     </row>
     <row r="46">
@@ -1902,7 +1902,7 @@
         </is>
       </c>
       <c r="E59" t="n">
-        <v>350</v>
+        <v>400</v>
       </c>
     </row>
     <row r="60">
@@ -2828,6 +2828,31 @@
       </c>
       <c r="E96" t="n">
         <v>280</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>CEDEVITA LIMUNSKA TRAVA</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>GAZIRANI I NEGAZIRANI SOKOVI</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>Pice</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>kom</t>
+        </is>
+      </c>
+      <c r="E97" t="n">
+        <v>150</v>
       </c>
     </row>
   </sheetData>

</xml_diff>